<commit_message>
Base de connaissances : arbitrages du 05/10 appliqués (fenêtres de semis, sol 10 °C, 90 jours entre engrais, profil sec, règles écrites dans la base)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/kb/Knowledge_et_cas_test_ENRICHI.xlsx
+++ b/docs/kb/Knowledge_et_cas_test_ENRICHI.xlsx
@@ -1,34 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones x Mois" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legende" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gazons Spécifiques" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objectifs Profil" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maladies &amp; Nuisibles" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Arrosage Précis" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pH &amp; Amendements" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tonte Précise" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cas de test" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cas de Test v3" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Règles Objectifs" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parcours Semis" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fenêtres Semis par Zone" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Température Sol &amp; ET0" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Règles Notifications" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Badges &amp; Objectifs" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEST - Nouveaux Modules" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEST - Couverture Notifs" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEST - KB Existante (audit)" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prépa Sol - Création" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prépa Sol - Regarnissage" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prépa Sol - Comparatif" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Zones x Mois" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Legende" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gazons Spécifiques" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Objectifs Profil" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Maladies &amp; Nuisibles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Arrosage Précis" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="pH &amp; Amendements" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Tonte Précise" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Cas de test" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Cas de Test v3" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Règles Objectifs" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Parcours Semis" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Fenêtres Semis par Zone" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Température Sol &amp; ET0" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Règles Notifications" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Badges &amp; Objectifs" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="TEST - Nouveaux Modules" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="TEST - Couverture Notifs" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="TEST - KB Existante (audit)" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Prépa Sol - Création" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Prépa Sol - Regarnissage" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Prépa Sol - Comparatif" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Règles complémentaires" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Journal" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Règles Objectifs'!$A$1:$G$38</definedName>
@@ -40,7 +42,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="57">
+  <fonts count="63">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -464,8 +466,41 @@
       <name val="Carlito"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1B5E20"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1B5E20"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FF555555"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="40">
+  <fills count="41">
     <fill>
       <patternFill/>
     </fill>
@@ -697,8 +732,13 @@
         <fgColor rgb="FFF4F8F4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1B5E20"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -839,6 +879,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBDBDBD"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBDBDBD"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBDBDBD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBDBDBD"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -850,7 +904,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="316">
+  <cellXfs count="325">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1789,6 +1843,27 @@
     <xf numFmtId="0" fontId="56" fillId="39" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="60" fillId="40" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="40" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2346,7 +2421,7 @@
       </c>
       <c r="P5" s="171" t="inlineStr">
         <is>
-          <t>Zone Nord-Est : uniquement mars (tmax requis ≥10°C). Autres zones : fév+mars possibles selon météo</t>
+          <t>Zones Nord-Est et Nord : uniquement mars (tmax requis ≥10°C). Autres zones : fév+mars possibles selon météo</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2567,7 @@
       </c>
       <c r="P8" s="171" t="inlineStr">
         <is>
-          <t>Mai-juin selon météo. Bloqué si sol détrempé (précip &gt;15mm). Délai min 45j depuis dernier engrais</t>
+          <t>Mai-juin selon météo. Bloqué si sol détrempé (précip &gt;15mm). Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -2752,7 +2827,7 @@
       </c>
       <c r="P13" s="171" t="inlineStr">
         <is>
-          <t>Septembre-octobre. Bloqué si gel ou sol détrempé. Délai 45j depuis dernier engrais</t>
+          <t>Septembre-octobre. Bloqué si gel ou sol détrempé. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2863,7 @@
       </c>
       <c r="P14" s="171" t="inlineStr">
         <is>
-          <t>Novembre uniquement. Potassium pour résistance au gel. Délai 45j depuis dernier engrais</t>
+          <t>Novembre uniquement. Potassium pour résistance au gel. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3303,7 @@
       </c>
       <c r="P23" s="171" t="inlineStr">
         <is>
-          <t>Mai-juin selon météo. Bloqué si sol détrempé (précip &gt;15mm). Délai min 45j depuis dernier engrais</t>
+          <t>Mai-juin selon météo. Bloqué si sol détrempé (précip &gt;15mm). Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -3488,7 +3563,7 @@
       </c>
       <c r="P28" s="171" t="inlineStr">
         <is>
-          <t>Septembre-octobre. Bloqué si gel ou sol détrempé. Délai 45j depuis dernier engrais</t>
+          <t>Septembre-octobre. Bloqué si gel ou sol détrempé. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -3524,7 +3599,7 @@
       </c>
       <c r="P29" s="171" t="inlineStr">
         <is>
-          <t>Novembre uniquement. Potassium pour résistance au gel. Délai 45j depuis dernier engrais</t>
+          <t>Novembre uniquement. Potassium pour résistance au gel. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -3964,7 +4039,7 @@
       </c>
       <c r="P38" s="171" t="inlineStr">
         <is>
-          <t>Mai-juin selon météo. Bloqué si sol détrempé (précip &gt;15mm). Délai min 45j depuis dernier engrais</t>
+          <t>Mai-juin selon météo. Bloqué si sol détrempé (précip &gt;15mm). Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -4224,7 +4299,7 @@
       </c>
       <c r="P43" s="171" t="inlineStr">
         <is>
-          <t>Septembre-octobre. Bloqué si gel ou sol détrempé. Délai 45j depuis dernier engrais</t>
+          <t>Septembre-octobre. Bloqué si gel ou sol détrempé. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -4260,7 +4335,7 @@
       </c>
       <c r="P44" s="171" t="inlineStr">
         <is>
-          <t>Novembre uniquement. Potassium pour résistance au gel. Délai 45j depuis dernier engrais</t>
+          <t>Novembre uniquement. Potassium pour résistance au gel. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -4696,7 +4771,7 @@
       </c>
       <c r="P53" s="171" t="inlineStr">
         <is>
-          <t>Mai-juin selon météo. Bloqué si sol détrempé (précip &gt;15mm). Délai min 45j depuis dernier engrais</t>
+          <t>Mai-juin selon météo. Bloqué si sol détrempé (précip &gt;15mm). Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -4956,7 +5031,7 @@
       </c>
       <c r="P58" s="171" t="inlineStr">
         <is>
-          <t>Septembre-octobre. Bloqué si gel ou sol détrempé. Délai 45j depuis dernier engrais</t>
+          <t>Septembre-octobre. Bloqué si gel ou sol détrempé. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -4992,7 +5067,7 @@
       </c>
       <c r="P59" s="171" t="inlineStr">
         <is>
-          <t>Novembre uniquement. Potassium pour résistance au gel. Délai 45j depuis dernier engrais</t>
+          <t>Novembre uniquement. Potassium pour résistance au gel. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -5282,7 +5357,7 @@
       </c>
       <c r="P65" s="171" t="inlineStr">
         <is>
-          <t>Zone Sud/Sud-Ouest : possible dès février. Toujours conditionné à tmax ≥8°C et pas de gel</t>
+          <t>Zone Nord : uniquement mars (tmax requis ≥10°C), comme le Nord-Est. Toujours conditionné à l'absence de gel</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5503,7 @@
       </c>
       <c r="P68" s="171" t="inlineStr">
         <is>
-          <t>Mai-juin selon météo. Bloqué si sol détrempé (précip &gt;15mm). Délai min 45j depuis dernier engrais</t>
+          <t>Mai-juin selon météo. Bloqué si sol détrempé (précip &gt;15mm). Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -5688,7 +5763,7 @@
       </c>
       <c r="P73" s="171" t="inlineStr">
         <is>
-          <t>Septembre-octobre. Bloqué si gel ou sol détrempé. Délai 45j depuis dernier engrais</t>
+          <t>Septembre-octobre. Bloqué si gel ou sol détrempé. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -5724,7 +5799,7 @@
       </c>
       <c r="P74" s="171" t="inlineStr">
         <is>
-          <t>Novembre uniquement. Potassium pour résistance au gel. Délai 45j depuis dernier engrais</t>
+          <t>Novembre uniquement. Potassium pour résistance au gel. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6235,7 @@
       </c>
       <c r="P83" s="171" t="inlineStr">
         <is>
-          <t>Mai-juin selon météo. Bloqué si sol détrempé (précip &gt;15mm). Délai min 45j depuis dernier engrais</t>
+          <t>Mai-juin selon météo. Bloqué si sol détrempé (précip &gt;15mm). Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -6420,7 +6495,7 @@
       </c>
       <c r="P88" s="171" t="inlineStr">
         <is>
-          <t>Septembre-octobre. Bloqué si gel ou sol détrempé. Délai 45j depuis dernier engrais</t>
+          <t>Septembre-octobre. Bloqué si gel ou sol détrempé. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6531,7 @@
       </c>
       <c r="P89" s="171" t="inlineStr">
         <is>
-          <t>Novembre uniquement. Potassium pour résistance au gel. Délai 45j depuis dernier engrais</t>
+          <t>Novembre uniquement. Potassium pour résistance au gel. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -6892,7 +6967,7 @@
       </c>
       <c r="P98" s="171" t="inlineStr">
         <is>
-          <t>Mai-juin selon météo. Bloqué si sol détrempé (précip &gt;15mm). Délai min 45j depuis dernier engrais</t>
+          <t>Mai-juin selon météo. Bloqué si sol détrempé (précip &gt;15mm). Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -7152,7 +7227,7 @@
       </c>
       <c r="P103" s="171" t="inlineStr">
         <is>
-          <t>Septembre-octobre. Bloqué si gel ou sol détrempé. Délai 45j depuis dernier engrais</t>
+          <t>Septembre-octobre. Bloqué si gel ou sol détrempé. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -7188,7 +7263,7 @@
       </c>
       <c r="P104" s="171" t="inlineStr">
         <is>
-          <t>Novembre uniquement. Potassium pour résistance au gel. Délai 45j depuis dernier engrais</t>
+          <t>Novembre uniquement. Potassium pour résistance au gel. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -9984,7 +10059,7 @@
       </c>
       <c r="D22" s="237" t="inlineStr">
         <is>
-          <t>Conditions standard (après J45)</t>
+          <t>Conditions standard (après J90)</t>
         </is>
       </c>
       <c r="E22" s="237" t="inlineStr">
@@ -9994,12 +10069,12 @@
       </c>
       <c r="F22" s="237" t="inlineStr">
         <is>
-          <t>Après J45</t>
+          <t>Après J90</t>
         </is>
       </c>
       <c r="G22" s="237" t="inlineStr">
         <is>
-          <t>OK si délai 45j depuis engrais précédent</t>
+          <t>OK si délai 90j depuis engrais précédent</t>
         </is>
       </c>
     </row>
@@ -10689,7 +10764,7 @@
       </c>
       <c r="C3" s="244" t="inlineStr">
         <is>
-          <t>Sol ≥ 10-12°C à 6cm (surveillance auto Open-Meteo)</t>
+          <t>Sol ≥ 10°C à 6cm (surveillance auto Open-Meteo)</t>
         </is>
       </c>
       <c r="D3" s="244" t="inlineStr">
@@ -10981,7 +11056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="153" min="1" max="1"/>
@@ -11071,7 +11146,7 @@
       </c>
       <c r="D4" s="250" t="inlineStr">
         <is>
-          <t>12°C</t>
+          <t>10°C</t>
         </is>
       </c>
       <c r="E4" s="251" t="inlineStr">
@@ -11118,7 +11193,7 @@
       </c>
       <c r="D5" s="250" t="inlineStr">
         <is>
-          <t>12°C</t>
+          <t>10°C</t>
         </is>
       </c>
       <c r="E5" s="251" t="inlineStr">
@@ -11212,7 +11287,7 @@
       </c>
       <c r="D7" s="250" t="inlineStr">
         <is>
-          <t>11°C</t>
+          <t>10°C</t>
         </is>
       </c>
       <c r="E7" s="251" t="inlineStr">
@@ -11397,7 +11472,7 @@
       </c>
       <c r="B13" s="254" t="inlineStr">
         <is>
-          <t>Sol 14°C (dans [12-25]) ✓ · pas de canicule sous 60j ✓ · établissement OK avant été</t>
+          <t>Sol 14°C (dans [10-25]) ✓ · pas de canicule sous 60j ✓ · établissement OK avant été</t>
         </is>
       </c>
       <c r="C13" s="255" t="n"/>
@@ -11443,7 +11518,7 @@
       </c>
       <c r="B15" s="254" t="inlineStr">
         <is>
-          <t>Sol 3°C &lt; min 12°C ✗</t>
+          <t>Sol 3°C &lt; min 10°C ✗</t>
         </is>
       </c>
       <c r="C15" s="255" t="n"/>
@@ -11513,6 +11588,13 @@
       <c r="A22" s="260" t="inlineStr">
         <is>
           <t>⚠️ Les mois affichés sont INDICATIFS (moyennes de zone). La décision réelle = toujours la température du sol Open-Meteo (soil_temperature_6cm) + trajectoire. Le pilotage par la donnée gère automatiquement les variations annuelles et micro-locales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="316" t="inlineStr">
+        <is>
+          <t>Dates retenues par l'app (05/10/2026) : la fenêtre s'ouvre au début indiqué (début = 1er, mi = 15, fin = 25) et se ferme à la fin indiquée (début = 10, mi = 15, fin = dernier jour du mois). Sol minimum 10 °C dans toutes les zones (décision du 05/10/2026).</t>
         </is>
       </c>
     </row>
@@ -11547,7 +11629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="153" min="1" max="2"/>
@@ -11615,7 +11697,7 @@
       </c>
       <c r="C3" s="244" t="inlineStr">
         <is>
-          <t>≥ 10-12°C</t>
+          <t>≥ 10°C</t>
         </is>
       </c>
       <c r="D3" s="244" t="inlineStr">
@@ -11825,7 +11907,44 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="154">
-      <c r="A10" s="261" t="inlineStr">
+      <c r="A10" s="317" t="inlineStr">
+        <is>
+          <t>Température sol 6cm</t>
+        </is>
+      </c>
+      <c r="B10" s="317" t="inlineStr">
+        <is>
+          <t>soil_temperature_6cm</t>
+        </is>
+      </c>
+      <c r="C10" s="317" t="inlineStr">
+        <is>
+          <t>≥ 8°C</t>
+        </is>
+      </c>
+      <c r="D10" s="317" t="inlineStr">
+        <is>
+          <t>Reprise de la pousse au printemps</t>
+        </is>
+      </c>
+      <c r="E10" s="317" t="inlineStr">
+        <is>
+          <t>Autorise la 1re tonte avant la date indicative de la zone</t>
+        </is>
+      </c>
+      <c r="F10" s="317" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="G10" s="317" t="inlineStr">
+        <is>
+          <t>Seuil de pousse (8 °C) distinct du seuil de semis (10 °C).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="261" t="inlineStr">
         <is>
           <t>PRINCIPE DE MATCHING : l'app utilise toujours l'info la plus précise DISPONIBLE. Ordre : station perso utilisateur &gt; Open-Meteo réel (Premium) &gt; estimation saisonnière (Gratuit). Ne jamais bloquer faute de donnée : fallback sur l'estimation.</t>
         </is>
@@ -11833,8 +11952,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A11:G11"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A10:G10"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -11848,7 +11967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="153" min="1" max="1"/>
@@ -11871,7 +11990,7 @@
     <row r="2" ht="42" customHeight="1" s="154">
       <c r="A2" s="262" t="inlineStr">
         <is>
-          <t>PRINCIPE : 1 notification/jour maximum (sauf urgence). Chaque jour, l'app envoie la source la plus prioritaire DISPONIBLE. Les niveaux 1-4 = contenu agronomique réel. Les niveaux 5-6 = filet de rétention les jours creux. Jamais de fausse urgence.</t>
+          <t>PRINCIPE : 2 notifications par jour au plus : le matin (l'action du jour) et, en saison d'arrosage, le soir (arrosage). Une urgence est toujours prioritaire. Sans notification autorisée, le même conseil part par email.</t>
         </is>
       </c>
     </row>
@@ -11930,7 +12049,7 @@
       </c>
       <c r="C4" s="244" t="inlineStr">
         <is>
-          <t>Gel imminent, canicule, pluie forte, seuils maladie atteints (voir onglet Maladies)</t>
+          <t>Gel imminent (tmin ≤ 2°C), canicule, pluie forte, seuils maladie atteints (voir onglet Maladies &amp; Nuisibles)</t>
         </is>
       </c>
       <c r="D4" s="244" t="inlineStr">
@@ -12172,14 +12291,14 @@
     <row r="11" ht="15" customHeight="1" s="154">
       <c r="A11" s="269" t="inlineStr">
         <is>
-          <t>RÈGLE ANTI-SPAM 1 : jamais plus d'1 notification programmée par jour (les urgences niveau 1 peuvent s'ajouter, rare).</t>
+          <t>RÈGLE ANTI-SPAM 1 : jamais plus de 2 notifications programmées par jour (créneau du matin + créneau du soir) ; l'urgence prend la place du message du créneau.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="154">
       <c r="A12" s="269" t="inlineStr">
         <is>
-          <t>RÈGLE ANTI-SPAM 2 : si l'utilisateur n'ouvre pas l'app après 5 notifs consécutives ignorées → réduire à 3x/semaine (anti-fatigue).</t>
+          <t>RÈGLE ANTI-SPAM 2 (anti-fatigue) : 7 jours sans visite → 1 notification par jour au plus, sans gamification ni astuce ; 21 jours → 2 à 3 par semaine. Urgences et parcours en cours exemptés.</t>
         </is>
       </c>
     </row>
@@ -12215,6 +12334,20 @@
       <c r="A18" s="271" t="inlineStr">
         <is>
           <t>RÈGLE N10 (cohérence arrosage, seuil 80%) : comparer le besoin en eau (ET₀ du jour) à la pluie prévue 24h. Si pluie ≥ 80% du besoin → arrosage ANNULÉ, message positif « pluie suffisante ✓ ». Si 20-80% → arrosage AJUSTÉ (« complétez X mm »). Si &lt; 20% → arrosage MAINTENU. La règle de départage est TOUJOURS quantitative (bilan hydrique), jamais un « il va pleuvoir » vague.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="318" t="inlineStr">
+        <is>
+          <t>RÈGLE RELANCE DES INACTIFS : à J+7, J+21 et J+45 sans visite (J+21 au minimum de novembre à février), 3 messages au plus par absence ; par notification, sinon par email. Retour mesuré = visite dans les 7 jours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="318" t="inlineStr">
+        <is>
+          <t>RÈGLE GEL : alerte « Gel cette nuit » si tmin ≤ 2°C ; les blocages d'actions (engrais, semis, arrosage) s'appliquent dès tmin &lt; 4°C.</t>
         </is>
       </c>
     </row>
@@ -12792,7 +12925,7 @@
       </c>
       <c r="C4" s="244" t="inlineStr">
         <is>
-          <t>Nord-Est, sol 11°C (min=12)</t>
+          <t>Nord-Est, sol 9°C (min=10)</t>
         </is>
       </c>
       <c r="D4" s="244" t="inlineStr">
@@ -12807,7 +12940,7 @@
       </c>
       <c r="F4" s="280" t="inlineStr">
         <is>
-          <t>SI soil_temp_6cm &lt; zone.seuil_min (Nord-Est=12°C) ALORS blocage + RDV. 11 &lt; 12 → bloqué.</t>
+          <t>SI soil_temp_6cm &lt; zone.seuil_min (10°C toutes zones) ALORS blocage + RDV. 9 &lt; 10 → bloqué.</t>
         </is>
       </c>
     </row>
@@ -12824,7 +12957,7 @@
       </c>
       <c r="C5" s="244" t="inlineStr">
         <is>
-          <t>Nord-Est, sol 12°C (min=12) + trajectoire OK</t>
+          <t>Nord-Est, sol 10°C (min=10) + trajectoire OK</t>
         </is>
       </c>
       <c r="D5" s="244" t="inlineStr">
@@ -12839,7 +12972,7 @@
       </c>
       <c r="F5" s="280" t="inlineStr">
         <is>
-          <t>Ouverture SI soil_temp_6cm &gt;= zone.seuil_min. 12 &gt;= 12 (Nord-Est) → autorisé (bornes incluses).</t>
+          <t>Ouverture SI soil_temp_6cm &gt;= zone.seuil_min. 10 &gt;= 10 → autorisé (bornes incluses).</t>
         </is>
       </c>
     </row>
@@ -12967,7 +13100,7 @@
       </c>
       <c r="F9" s="280" t="inlineStr">
         <is>
-          <t>SI soil_temp_6cm &lt; zone.seuil_min. Nord-Est 3 &lt; 12 → bloqué. RDV = 1er jour où soil_temp prévu &gt;= 12°C (estimation ~mi-avril).</t>
+          <t>SI soil_temp_6cm &lt; zone.seuil_min. Nord-Est 3 &lt; 10 → bloqué. RDV = 1er jour où soil_temp prévu &gt;= 10°C (estimation ~mi-avril).</t>
         </is>
       </c>
     </row>
@@ -14008,12 +14141,12 @@
       </c>
       <c r="C42" s="244" t="inlineStr">
         <is>
-          <t>5 notifs consécutives ignorées</t>
+          <t>7 jours sans visite dans l'app</t>
         </is>
       </c>
       <c r="D42" s="244" t="inlineStr">
         <is>
-          <t>Réduction auto à 3x/semaine</t>
+          <t>1 notification par jour au plus, sans gamification ni astuce ; 21 jours → 2 à 3 par semaine</t>
         </is>
       </c>
       <c r="E42" s="279" t="inlineStr">
@@ -14023,7 +14156,7 @@
       </c>
       <c r="F42" s="280" t="inlineStr">
         <is>
-          <t>SI notifs_ignorees_consecutives &gt;= 5 ALORS fréquence_max = 3/semaine (mode anti-fatigue) jusqu'à réouverture.</t>
+          <t>SI jours_sans_visite &gt;= 7 ALORS 1/jour (urgences et parcours exemptés) ; SI &gt;= 21 ALORS 2-3/semaine.</t>
         </is>
       </c>
     </row>
@@ -15627,7 +15760,7 @@
       </c>
       <c r="E7" s="280" t="inlineStr">
         <is>
-          <t>Seuils AIR (lawn.js) : gel temp_min&lt;=2, canicule temp_max&gt;=33. Seuil SOL (&gt;=10-12°C) = NOUVEAU, à ajouter pour le semis via Open-Meteo. Pas de conflit : air=entretien, sol=semis.</t>
+          <t>Seuils AIR (lawn.js) : gel temp_min&lt;=2, canicule temp_max&gt;=33. Seuil SOL (&gt;=10°C) = semis (10 °C). Pas de conflit : air=entretien, sol=semis.</t>
         </is>
       </c>
       <c r="F7" s="298" t="inlineStr">
@@ -17906,7 +18039,7 @@
       </c>
       <c r="B15" s="175" t="inlineStr">
         <is>
-          <t>Bloqué si appliqué il y a &lt; 90 jours</t>
+          <t>Bloqué si appliqué il y a &lt; 90 jours (1 engrais par saison, 4 par an au plus)</t>
         </is>
       </c>
     </row>
@@ -18002,7 +18135,7 @@
       </c>
       <c r="B24" s="176" t="inlineStr">
         <is>
-          <t>tmin &lt; 4°C — bloque engrais, semences, biostimulant, arrosage</t>
+          <t>tmin &lt; 4°C — bloque engrais, semences, biostimulant, arrosage · alerte « Gel cette nuit » (notification d'urgence) si tmin ≤ 2°C</t>
         </is>
       </c>
     </row>
@@ -18026,7 +18159,7 @@
       </c>
       <c r="B26" s="176" t="inlineStr">
         <is>
-          <t>précip &gt; 3mm — bloque désherbage et scarification</t>
+          <t>précip &gt; 3mm — bloque désherbage et scarification · précip &gt; 5mm — bloque la tonte</t>
         </is>
       </c>
     </row>
@@ -19193,13 +19326,349 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" style="154" min="1" max="1"/>
+    <col width="38" customWidth="1" style="154" min="2" max="2"/>
+    <col width="110" customWidth="1" style="154" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="319" t="inlineStr">
+        <is>
+          <t>➕ MONGAZON360 — Règles complémentaires (validées le 05/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="320" t="inlineStr">
+        <is>
+          <t>Règles appliquées par l'app qui complètent les autres onglets. Elles font partie de la base au même titre que les autres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="321" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="B4" s="321" t="inlineStr">
+        <is>
+          <t>Règle</t>
+        </is>
+      </c>
+      <c r="C4" s="321" t="inlineStr">
+        <is>
+          <t>Valeur</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="322" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="323" t="inlineStr">
+        <is>
+          <t>Date indicative de 1re tonte par zone</t>
+        </is>
+      </c>
+      <c r="C5" s="322" t="inlineStr">
+        <is>
+          <t>Sud et Corse 1er mars · Sud-Ouest 10 mars · Ouest 15 mars · Centre 20 mars · Nord 25 mars · Nord-Est 1er avril. Plus tôt si le sol atteint 8 °C (pousse).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="322" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="323" t="inlineStr">
+        <is>
+          <t>Hauteur de la 1re tonte</t>
+        </is>
+      </c>
+      <c r="C6" s="322" t="inlineStr">
+        <is>
+          <t>En haut de la fourchette de printemps du gazon : 6 cm pour un gazon universel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="322" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="323" t="inlineStr">
+        <is>
+          <t>Calendrier de reprise du printemps</t>
+        </is>
+      </c>
+      <c r="C7" s="322" t="inlineStr">
+        <is>
+          <t>Révision de la tondeuse 3 semaines avant la 1re tonte · scarification 2 semaines après · regarnissage et engrais de démarrage juste après la scarification, jamais avant la fenêtre de semis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="322" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="323" t="inlineStr">
+        <is>
+          <t>Notification « Premières gelées en vue »</t>
+        </is>
+      </c>
+      <c r="C8" s="322" t="inlineStr">
+        <is>
+          <t>Octobre à décembre, minimum entre 3 et 5 °C : purger l'arrosage automatique, ou ranger tuyau et arroseur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="322" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="323" t="inlineStr">
+        <is>
+          <t>Notification « Ramasse les feuilles »</t>
+        </is>
+      </c>
+      <c r="C9" s="322" t="inlineStr">
+        <is>
+          <t>Octobre à décembre, jour sec (pluie &lt; 1 mm, vent &lt; 30 km/h), au plus tous les 14 jours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="322" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="323" t="inlineStr">
+        <is>
+          <t>Notification « Dernière tonte »</t>
+        </is>
+      </c>
+      <c r="C10" s="322" t="inlineStr">
+        <is>
+          <t>Novembre, jour sec, au moins 10 °C, à 5-6 cm (pas pour un robot).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="322" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="323" t="inlineStr">
+        <is>
+          <t>Notification « Mesure le pH »</t>
+        </is>
+      </c>
+      <c r="C11" s="322" t="inlineStr">
+        <is>
+          <t>Du 1er au 12 octobre, hors sol calcaire : chaulage d'automne si pH &lt; 6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="322" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="323" t="inlineStr">
+        <is>
+          <t>Notifications de reprise</t>
+        </is>
+      </c>
+      <c r="C12" s="322" t="inlineStr">
+        <is>
+          <t>Révision de la tondeuse (ou du robot) de J-21 à J-14 avant la 1re tonte ; « C'est le moment de la 1re tonte » de J-3 à J+7 si sec et au moins 10 °C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="322" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="323" t="inlineStr">
+        <is>
+          <t>Astuces d'hiver</t>
+        </is>
+      </c>
+      <c r="C13" s="322" t="inlineStr">
+        <is>
+          <t>Taupinières : étaler au râteau · neige : laisser fondre, ne pas tasser · flaques : noter les zones à aérer au printemps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="322" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="323" t="inlineStr">
+        <is>
+          <t>Kits de saison</t>
+        </is>
+      </c>
+      <c r="C14" s="322" t="inlineStr">
+        <is>
+          <t>Produits de saison du mois pour la zone (matrice Zones x Mois), 4 au plus ; semences et anti-mousse comptés sur ~30 % de la surface ; scarificateur OU aérateur ; pas de NPK de synthèse en objectif naturel ; pas de chaux sur sol calcaire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="322" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="323" t="inlineStr">
+        <is>
+          <t>Diagnostic photo d'hiver</t>
+        </is>
+      </c>
+      <c r="C15" s="322" t="inlineStr">
+        <is>
+          <t>Novembre à février : repos hivernal non pénalisé ; recherche de mousse, fusariose / moisissure des neiges, taupinières, eau stagnante, feuilles, traces de gel ; pas d'engrais azoté en hiver.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="322" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="323" t="inlineStr">
+        <is>
+          <t>Conformité phytosanitaire</t>
+        </is>
+      </c>
+      <c r="C16" s="322" t="inlineStr">
+        <is>
+          <t>Jamais de fongicide ni de désherbant chimique conseillé (loi Labbé) : prévention, gestes mécaniques, biocontrôle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="322" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="323" t="inlineStr">
+        <is>
+          <t>Espacement chaulage / engrais / sulfate de fer</t>
+        </is>
+      </c>
+      <c r="C17" s="322" t="inlineStr">
+        <is>
+          <t>Au moins 3 à 4 semaines entre un chaulage et un engrais azoté ou un anti-mousse au sulfate de fer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="322" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="323" t="inlineStr">
+        <is>
+          <t>Relance des inactifs</t>
+        </is>
+      </c>
+      <c r="C18" s="322" t="inlineStr">
+        <is>
+          <t>J+7, J+21, J+45 sans visite (J+21 au minimum de novembre à février), 3 messages au plus par absence, notification sinon email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="322" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="323" t="inlineStr">
+        <is>
+          <t>Anti-fatigue</t>
+        </is>
+      </c>
+      <c r="C19" s="322" t="inlineStr">
+        <is>
+          <t>7 jours sans visite → 1 notification par jour, sans gamification ni astuce ; 21 jours → 2 à 3 par semaine ; urgences et parcours exemptés.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" style="154" min="1" max="1"/>
+    <col width="130" customWidth="1" style="154" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="319" t="inlineStr">
+        <is>
+          <t>📝 Journal des évolutions de la base</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="324" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B3" s="324" t="inlineStr">
+        <is>
+          <t>Évolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="153" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="B4" s="318" t="inlineStr">
+        <is>
+          <t>Base ajoutée au dépôt de l'app (docs/kb) ; règle : toute information donnée aux utilisateurs vient de la base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="153" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="318" t="inlineStr">
+        <is>
+          <t>Arbitrages : fenêtres de semis de la base appliquées par l'app, sol minimum 10 °C partout (seuil de pousse 8 °C pour la 1re tonte) ; engrais de démarrage en mars seulement en Nord et Nord-Est ; 90 jours entre deux engrais (1 par saison, 4 par an au plus) ; profil « sec » → Rustique, « chaud » → Bermuda ; fongicides chimiques retirés ; règles de notification, gel (≤ 2 °C) et pluie/tonte (&gt; 5 mm) écrites ; onglet « Règles complémentaires » (15 règles validées).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.73046875" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="153" min="1" max="1"/>
@@ -19806,6 +20275,13 @@
         <is>
           <t>Voir KB principale
 (Cas de test)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="316" t="inlineStr">
+        <is>
+          <t>Profils de l'app (05/10/2026) : « Sec / méditerranéen » → règles Rustique · « Gazon chaud » → règles Bermuda · « Je ne sais pas » → Universel.</t>
         </is>
       </c>
     </row>
@@ -20235,7 +20711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.73046875" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="153" min="1" max="1"/>
@@ -20380,15 +20856,15 @@
       </c>
       <c r="J4" s="201" t="inlineStr">
         <is>
-          <t>Fongicide préventif
-autonme + printemps
-(iprodione, thirame)</t>
+          <t>Éviter l'azote en fin d'automne,
+aérer, ramasser les feuilles,
+ne pas tondre trop ras</t>
         </is>
       </c>
       <c r="K4" s="201" t="inlineStr">
         <is>
-          <t>Fongicide systémique
-immédiat</t>
+          <t>Biocontrôle ou
+professionnel agréé</t>
         </is>
       </c>
       <c r="L4" s="201" t="inlineStr">
@@ -20459,8 +20935,7 @@
       </c>
       <c r="K5" s="203" t="inlineStr">
         <is>
-          <t>Fongicide à base
-de soufre</t>
+          <t>Soufre (biocontrôle)</t>
         </is>
       </c>
       <c r="L5" s="203" t="inlineStr">
@@ -20530,8 +21005,8 @@
       </c>
       <c r="K6" s="199" t="inlineStr">
         <is>
-          <t>Fongicide
-(chlorothalonil)</t>
+          <t>Biocontrôle ou
+professionnel agréé</t>
         </is>
       </c>
       <c r="L6" s="199" t="inlineStr">
@@ -20601,8 +21076,8 @@
       </c>
       <c r="K7" s="206" t="inlineStr">
         <is>
-          <t>Fongicide spécifique
-(métalaxyl)</t>
+          <t>Biocontrôle ou
+professionnel agréé</t>
         </is>
       </c>
       <c r="L7" s="206" t="inlineStr">
@@ -20672,8 +21147,8 @@
       </c>
       <c r="K8" s="208" t="inlineStr">
         <is>
-          <t>Fongicide
-(propiconazole)</t>
+          <t>Biocontrôle ou
+professionnel agréé</t>
         </is>
       </c>
       <c r="L8" s="208" t="inlineStr">
@@ -20742,8 +21217,8 @@
       </c>
       <c r="K9" s="210" t="inlineStr">
         <is>
-          <t>Fongicide
-(triazole)</t>
+          <t>Biocontrôle ou
+professionnel agréé</t>
         </is>
       </c>
       <c r="L9" s="210" t="inlineStr">
@@ -21264,6 +21739,13 @@
         <is>
           <t>Cycle 3-4 ans
 selon espèce</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="316" t="inlineStr">
+        <is>
+          <t>Règle générale (05/10/2026) : l'app, Bob, le diagnostic et les articles ne conseillent jamais de fongicide ni de désherbant chimique (loi Labbé) : prévention, gestes mécaniques et biocontrôle uniquement ; au-delà, recours à un professionnel agréé.</t>
         </is>
       </c>
     </row>
@@ -22932,7 +23414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.73046875" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="153" min="1" max="1"/>
@@ -23624,6 +24106,13 @@
           <t>Scalpage visible,
 jaunissement,
 mauvaises herbes++</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="316" t="inlineStr">
+        <is>
+          <t>Profils de l'app (05/10/2026) : « Sec / méditerranéen » → règles Rustique · « Gazon chaud » → règles Bermuda · « Je ne sais pas » → Universel.</t>
         </is>
       </c>
     </row>
@@ -24115,7 +24604,7 @@
       </c>
       <c r="M8" s="175" t="inlineStr">
         <is>
-          <t>Engrais il y a 30j (&lt;45j)</t>
+          <t>Engrais il y a 30j (&lt;90j)</t>
         </is>
       </c>
       <c r="N8" s="228" t="inlineStr">
@@ -24169,7 +24658,7 @@
       </c>
       <c r="K9" s="225" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>100j</t>
         </is>
       </c>
       <c r="L9" s="226" t="inlineStr">
@@ -24179,7 +24668,7 @@
       </c>
       <c r="M9" s="175" t="inlineStr">
         <is>
-          <t>Engrais il y a 50j (≥45j)</t>
+          <t>Engrais il y a 100j (≥90j)</t>
         </is>
       </c>
       <c r="N9" s="228" t="inlineStr">
@@ -25331,7 +25820,7 @@
       </c>
       <c r="M27" s="175" t="inlineStr">
         <is>
-          <t>Engrais il y a 30j (&lt;45j)</t>
+          <t>Engrais il y a 30j (&lt;90j)</t>
         </is>
       </c>
       <c r="N27" s="228" t="inlineStr">
@@ -26935,7 +27424,7 @@
       </c>
       <c r="M52" s="175" t="inlineStr">
         <is>
-          <t>Engrais il y a 30j (&lt;45j)</t>
+          <t>Engrais il y a 30j (&lt;90j)</t>
         </is>
       </c>
       <c r="N52" s="228" t="inlineStr">

</xml_diff>

<commit_message>
Engrais d'hiver : exception de 45 jours après l'engrais d'automne (base et app)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/kb/Knowledge_et_cas_test_ENRICHI.xlsx
+++ b/docs/kb/Knowledge_et_cas_test_ENRICHI.xlsx
@@ -2863,7 +2863,7 @@
       </c>
       <c r="P14" s="171" t="inlineStr">
         <is>
-          <t>Novembre uniquement. Potassium pour résistance au gel. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
+          <t>Novembre uniquement. Potassium pour résistance au gel. Exception : 45j minimum après l'engrais d'automne (90j après tout autre engrais)</t>
         </is>
       </c>
     </row>
@@ -3599,7 +3599,7 @@
       </c>
       <c r="P29" s="171" t="inlineStr">
         <is>
-          <t>Novembre uniquement. Potassium pour résistance au gel. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
+          <t>Novembre uniquement. Potassium pour résistance au gel. Exception : 45j minimum après l'engrais d'automne (90j après tout autre engrais)</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="P44" s="171" t="inlineStr">
         <is>
-          <t>Novembre uniquement. Potassium pour résistance au gel. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
+          <t>Novembre uniquement. Potassium pour résistance au gel. Exception : 45j minimum après l'engrais d'automne (90j après tout autre engrais)</t>
         </is>
       </c>
     </row>
@@ -5067,7 +5067,7 @@
       </c>
       <c r="P59" s="171" t="inlineStr">
         <is>
-          <t>Novembre uniquement. Potassium pour résistance au gel. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
+          <t>Novembre uniquement. Potassium pour résistance au gel. Exception : 45j minimum après l'engrais d'automne (90j après tout autre engrais)</t>
         </is>
       </c>
     </row>
@@ -5799,7 +5799,7 @@
       </c>
       <c r="P74" s="171" t="inlineStr">
         <is>
-          <t>Novembre uniquement. Potassium pour résistance au gel. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
+          <t>Novembre uniquement. Potassium pour résistance au gel. Exception : 45j minimum après l'engrais d'automne (90j après tout autre engrais)</t>
         </is>
       </c>
     </row>
@@ -6531,7 +6531,7 @@
       </c>
       <c r="P89" s="171" t="inlineStr">
         <is>
-          <t>Novembre uniquement. Potassium pour résistance au gel. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
+          <t>Novembre uniquement. Potassium pour résistance au gel. Exception : 45j minimum après l'engrais d'automne (90j après tout autre engrais)</t>
         </is>
       </c>
     </row>
@@ -7263,7 +7263,7 @@
       </c>
       <c r="P104" s="171" t="inlineStr">
         <is>
-          <t>Novembre uniquement. Potassium pour résistance au gel. Délai min 90j depuis le dernier engrais (1 par saison, 4 par an au plus)</t>
+          <t>Novembre uniquement. Potassium pour résistance au gel. Exception : 45j minimum après l'engrais d'automne (90j après tout autre engrais)</t>
         </is>
       </c>
     </row>
@@ -7429,6 +7429,7 @@
         </is>
       </c>
     </row>
+    <row r="108"/>
     <row r="109" ht="18" customHeight="1" s="154">
       <c r="A109" s="172" t="inlineStr">
         <is>
@@ -18039,7 +18040,7 @@
       </c>
       <c r="B15" s="175" t="inlineStr">
         <is>
-          <t>Bloqué si appliqué il y a &lt; 90 jours (1 engrais par saison, 4 par an au plus)</t>
+          <t>Bloqué si appliqué il y a &lt; 90 jours (1 engrais par saison, 4 par an au plus) · exception : engrais d'hiver possible 45 jours après l'engrais d'automne</t>
         </is>
       </c>
     </row>
@@ -19607,7 +19608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="154" min="1" max="1"/>
@@ -19654,6 +19655,18 @@
       <c r="B5" s="318" t="inlineStr">
         <is>
           <t>Arbitrages : fenêtres de semis de la base appliquées par l'app, sol minimum 10 °C partout (seuil de pousse 8 °C pour la 1re tonte) ; engrais de démarrage en mars seulement en Nord et Nord-Est ; 90 jours entre deux engrais (1 par saison, 4 par an au plus) ; profil « sec » → Rustique, « chaud » → Bermuda ; fongicides chimiques retirés ; règles de notification, gel (≤ 2 °C) et pluie/tonte (&gt; 5 mm) écrites ; onglet « Règles complémentaires » (15 règles validées).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Exception : engrais d'hiver (novembre) autorisé 45 jours après l'engrais d'automne, pour garder 4 engrais par an.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tonte bloquée sur herbe ou sol mouillés (correctif urgent)
Tonte bloquée un jour de pluie (code météo ≥ 51), dès 2 mm prévus ou après plus de
10 mm la veille, au lieu de « plus de 5 mm » : actions du jour, proposition du robot,
rappels de tonte (qui ignoraient la pluie) et consignes de Bob. Pluie de la veille
ajoutée à la météo (past_days=1, retirée des séries). Seuils dans tonteGazon.json ;
base de connaissances mise à jour (Règles complémentaires n° 16, Légende, Journal).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/kb/Knowledge_et_cas_test_ENRICHI.xlsx
+++ b/docs/kb/Knowledge_et_cas_test_ENRICHI.xlsx
@@ -7429,7 +7429,6 @@
         </is>
       </c>
     </row>
-    <row r="108"/>
     <row r="109" ht="18" customHeight="1" s="154">
       <c r="A109" s="172" t="inlineStr">
         <is>
@@ -18160,7 +18159,7 @@
       </c>
       <c r="B26" s="176" t="inlineStr">
         <is>
-          <t>précip &gt; 3mm — bloque désherbage et scarification · précip &gt; 5mm — bloque la tonte</t>
+          <t>précip &gt; 3mm — bloque désherbage et scarification · tonte : voir « Pluie et tonte » (Règles complémentaires)</t>
         </is>
       </c>
     </row>
@@ -19333,7 +19332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="154" min="1" max="1"/>
@@ -19582,7 +19581,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" s="154">
       <c r="A19" s="322" t="n">
         <v>15</v>
       </c>
@@ -19594,6 +19593,21 @@
       <c r="C19" s="322" t="inlineStr">
         <is>
           <t>7 jours sans visite → 1 notification par jour, sans gamification ni astuce ; 21 jours → 2 à 3 par semaine ; urgences et parcours exemptés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" s="154">
+      <c r="A20" s="322" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="323" t="inlineStr">
+        <is>
+          <t>Pluie et tonte</t>
+        </is>
+      </c>
+      <c r="C20" s="322" t="inlineStr">
+        <is>
+          <t>Tonte bloquée sur herbe ou sol mouillés : jour de pluie (code météo du jour ≥ 51 : bruine, pluie, neige, averses, orage, quelle que soit la quantité), ou ≥ 2 mm de pluie prévus dans la journée, ou &gt; 10 mm tombés la veille (sol détrempé). S'applique aux actions du jour, aux rappels, à Bob et à la mise au repos proposée du robot. Remplace l'ancien seuil « &gt; 5 mm ».</t>
         </is>
       </c>
     </row>
@@ -19608,7 +19622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="154" min="1" max="1"/>
@@ -19658,15 +19672,27 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" s="154">
+      <c r="A6" s="153" t="inlineStr">
         <is>
           <t>05/10/2026</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="153" t="inlineStr">
         <is>
           <t>Exception : engrais d'hiver (novembre) autorisé 45 jours après l'engrais d'automne, pour garder 4 engrais par an.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" s="154">
+      <c r="A7" s="153" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="153" t="inlineStr">
+        <is>
+          <t>Pluie et tonte : tonte bloquée un jour de pluie, dès 2 mm prévus ou après plus de 10 mm la veille (au lieu de &gt; 5 mm), validé par Jordan après une tonte proposée sous la pluie (4,3 mm).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Arrosage : pluie de la veille déduite (correctif urgent)
La pluie de la veille compte avec celle du jour : arrosage supprimé dès 8 mm cumulés,
dose réduite au-delà de 2 ou 5 mm (calcArrosage, plan, recommandations, semaine,
arrosage connecté). Semis et regarnissage : la moitié de la pluie de la veille est
déduite du besoin. Prochain arrosage affiché « Demain, selon la météo ». Base de
connaissances : Règles complémentaires n° 17 et Journal.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/kb/Knowledge_et_cas_test_ENRICHI.xlsx
+++ b/docs/kb/Knowledge_et_cas_test_ENRICHI.xlsx
@@ -19332,7 +19332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="154" min="1" max="1"/>
@@ -19608,6 +19608,21 @@
       <c r="C20" s="322" t="inlineStr">
         <is>
           <t>Tonte bloquée sur herbe ou sol mouillés : jour de pluie (code météo du jour ≥ 51 : bruine, pluie, neige, averses, orage, quelle que soit la quantité), ou ≥ 2 mm de pluie prévus dans la journée, ou &gt; 10 mm tombés la veille (sol détrempé). S'applique aux actions du jour, aux rappels, à Bob et à la mise au repos proposée du robot. Remplace l'ancien seuil « &gt; 5 mm ».</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" s="154">
+      <c r="A21" s="322" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="323" t="inlineStr">
+        <is>
+          <t>Pluie et arrosage</t>
+        </is>
+      </c>
+      <c r="C21" s="322" t="inlineStr">
+        <is>
+          <t>La pluie de la veille compte avec celle du jour : arrosage supprimé si leur total atteint 8 mm (10 mm pour le calcul de dose), dose réduite au-delà de 2 mm (−50 %) ou 5 mm (−80 % du cumul). Semis et regarnissage (micro-arrosages) : déficit = ET₀ − pluie du jour − la moitié de la pluie de la veille (la surface sèche vite). Le prochain arrosage annoncé reste à confirmer le jour même selon la météo.</t>
         </is>
       </c>
     </row>
@@ -19622,7 +19637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="154" min="1" max="1"/>
@@ -19693,6 +19708,18 @@
       <c r="B7" s="153" t="inlineStr">
         <is>
           <t>Pluie et tonte : tonte bloquée un jour de pluie, dès 2 mm prévus ou après plus de 10 mm la veille (au lieu de &gt; 5 mm), validé par Jordan après une tonte proposée sous la pluie (4,3 mm).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" s="154">
+      <c r="A8" s="153" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="153" t="inlineStr">
+        <is>
+          <t>Pluie et arrosage : la pluie de la veille est déduite de l'arrosage du jour (classique, semis, regarnissage, arrosage connecté), validé par Jordan.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diagnostic de suivi : règle validée par Jordan ajoutée à la base de connaissances (Règles complémentaires n° 18)
30 jours après une scarification = moment de la photo de suivi (précision de Jordan du 19/10, pas un point à faire
d'ici le 17/11) : journal corrigé, source de suiviDiagnostic.json et commentaire de la recette n° 54 alignés.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/kb/Knowledge_et_cas_test_ENRICHI.xlsx
+++ b/docs/kb/Knowledge_et_cas_test_ENRICHI.xlsx
@@ -19474,7 +19474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="154" min="1" max="1"/>
@@ -19765,6 +19765,21 @@
       <c r="C21" s="322" t="inlineStr">
         <is>
           <t>La pluie de la veille compte avec celle du jour : arrosage supprimé si leur total atteint 8 mm (10 mm pour le calcul de dose), dose réduite au-delà de 2 mm (−50 %) ou 5 mm (−80 % du cumul). Semis et regarnissage (micro-arrosages) : déficit = ET₀ − pluie du jour − la moitié de la pluie de la veille (la surface sèche vite). Le prochain arrosage annoncé reste à confirmer le jour même selon la météo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="322" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="323" t="inlineStr">
+        <is>
+          <t>Diagnostic de suivi (avant / après)</t>
+        </is>
+      </c>
+      <c r="C22" s="322" t="inlineStr">
+        <is>
+          <t>Sur la page Diagnostic uniquement : après un diagnostic, l'utilisateur indique les travaux faits dans les 45 jours (regarnissage, scarification, anti-mousse, désherbage) et leur date. Une photo du même endroit est proposée pendant 7 jours, 30 jours après un regarnissage (levée J21-J45, onglet Parcours Semis), une scarification ou un anti-mousse, 21 jours après un désherbage (délais entre deux traitements, onglet Legende) ; plusieurs travaux → le délai le plus long. Elle est comparée au diagnostic des travaux si elle est prise entre 7 jours avant et 30 jours après cette date : écart de score, problèmes réglés, encore là ou nouveaux. Pas de notification ; rien pendant l'essai de 7 jours.</t>
         </is>
       </c>
     </row>
@@ -20084,7 +20099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="154" min="1" max="1"/>
@@ -20191,6 +20206,18 @@
       <c r="B10" s="153" t="inlineStr">
         <is>
           <t>Ajout validé par Jordan : capteurs du jardin (onglet « Température Sol &amp; ET0 ») : humidité du sol mesurée (seuils FAO-56 par type de sol, sol humide → pas d'arrosage, sol sec → arrosage conseillé, ignorée pendant un semis) et température du sol mesurée (remplace l'estimation du jour).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="153" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="153" t="inlineStr">
+        <is>
+          <t>Ajout validé par Jordan : diagnostic de suivi (« Règles complémentaires » n° 18) : photo du même endroit 30 jours après un regarnissage, une scarification ou un anti-mousse, 21 jours après un désherbage, comparée au diagnostic des travaux.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ligue d'hiver : départage décidé par Jordan (accès Premium, puis compte le plus ancien) ; badge et notifications dans la base
Règlement (CGU 6 g) : en cas d'égalité, un compte avec l'accès Premium (abonnement, essai ou Premium offert) passe devant
un compte gratuit, puis le compte le plus ancien ; plus de tirage au sort. Participants comme proposé (décision du 20/10).
Pilotage → Activité classe les plus assidus dans cet ordre. Base de connaissances : badge « Gardien de l'hiver »
(Badges & Objectifs) et règle de notification de la ligue (Règles Notifications), validés par Jordan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/kb/Knowledge_et_cas_test_ENRICHI.xlsx
+++ b/docs/kb/Knowledge_et_cas_test_ENRICHI.xlsx
@@ -11998,7 +11998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="153" min="1" max="1"/>
@@ -12319,6 +12319,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="154">
       <c r="A11" s="269" t="inlineStr">
         <is>
@@ -12354,6 +12355,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="43.5" customHeight="1" s="154">
       <c r="A17" s="271" t="inlineStr">
         <is>
@@ -12379,6 +12381,13 @@
       <c r="A20" s="318" t="inlineStr">
         <is>
           <t>RÈGLE GEL : alerte « Gel cette nuit » si tmin ≤ 2°C ; les blocages d'actions (engrais, semis, arrosage) s'appliquent dès tmin &lt; 4°C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="318" t="inlineStr">
+        <is>
+          <t>RÈGLE LIGUE D'HIVER (validée le 20/10/2026) : du 1er novembre au 30 janvier, quiz du dimanche (le dimanche, sinon les jours suivants tant qu'il n'est pas fait) et défi de la semaine (à partir du mercredi s'il n'est pas fait) en niveau 5, une fois par semaine chacun ; les réponses expliquées des quiz passés rejoignent les astuces du niveau 6 (« Le savais-tu ? »). Rythme inchangé : une notification le matin au plus, anti-fatigue appliquée.</t>
         </is>
       </c>
     </row>
@@ -12406,7 +12415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="24" customWidth="1" style="153" min="1" max="1"/>
@@ -12838,29 +12847,67 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1" s="154">
-      <c r="A15" s="277" t="inlineStr">
-        <is>
-          <t>RÈGLE RARETÉ : ne jamais descendre en dessous de l'exigence. Un badge facile à obtenir perd toute valeur.</t>
-        </is>
-      </c>
-    </row>
+    <row r="14" ht="48" customHeight="1" s="154">
+      <c r="A14" s="243" t="inlineStr">
+        <is>
+          <t>❄️ Gardien de l'hiver [année]</t>
+        </is>
+      </c>
+      <c r="B14" s="276" t="inlineStr">
+        <is>
+          <t>Saisonnier</t>
+        </is>
+      </c>
+      <c r="C14" s="244" t="inlineStr">
+        <is>
+          <t>Relever au moins 10 semaines sur 13 de la Ligue d'hiver (défi et quiz de la semaine faits la même semaine)</t>
+        </is>
+      </c>
+      <c r="D14" s="244" t="inlineStr">
+        <is>
+          <t>Gratuit</t>
+        </is>
+      </c>
+      <c r="E14" s="244" t="inlineStr">
+        <is>
+          <t>🟣 Édition limitée</t>
+        </is>
+      </c>
+      <c r="F14" s="244" t="inlineStr">
+        <is>
+          <t>Gardien de l'hiver [année] ! Badge non reconductible ❄️</t>
+        </is>
+      </c>
+      <c r="G14" s="244" t="inlineStr">
+        <is>
+          <t>Rendez-vous hebdomadaire de l'hiver = anti-churn</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" s="154"/>
     <row r="16" ht="30" customHeight="1" s="154">
       <c r="A16" s="277" t="inlineStr">
         <is>
+          <t>RÈGLE RARETÉ : ne jamais descendre en dessous de l'exigence. Un badge facile à obtenir perd toute valeur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1" s="154">
+      <c r="A17" s="277" t="inlineStr">
+        <is>
           <t>PAS DE POINTS BONUS : les badges sont symboliques. Les actions du parcours rapportent leur barème GreenPoints NORMAL (le cumul vient du volume, déjà mesuré par actions7j/14j/30j dans lawnScore).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1" s="154">
-      <c r="A17" s="259" t="inlineStr">
-        <is>
-          <t>BADGES SAISONNIERS : millésimés ([année]) et non reconductibles. « Champion du Printemps 2027 » ne pourra plus jamais être obtenu après = collection + rendez-vous annuel = antidote au churn saisonnier.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1" s="154">
       <c r="A18" s="259" t="inlineStr">
+        <is>
+          <t>BADGES SAISONNIERS : millésimés ([année]) et non reconductibles. « Champion du Printemps 2027 » ne pourra plus jamais être obtenu après = collection + rendez-vous annuel = antidote au churn saisonnier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1" s="154">
+      <c r="A19" s="259" t="inlineStr">
         <is>
           <t>ÉVOLUTIF : commencer avec ces ~10 badges. En ajouter seulement si un accomplissement réellement rare et non couvert émerge (ex. premier objet connecté relié, quand les API seront actives).</t>
         </is>
@@ -12873,7 +12920,7 @@
     <mergeCell ref="A18:G18"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A16:G16"/>
-    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A19:G19"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -19973,7 +20020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="154" min="1" max="1"/>
@@ -19987,6 +20034,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="324" t="inlineStr">
         <is>
@@ -20068,6 +20116,18 @@
       <c r="B9" s="153" t="inlineStr">
         <is>
           <t>Ajout validé par Jordan : onglet « Sujets complémentaires » (champignons et ronds de sorcière, gazon en plaques, mulching), pour les articles Conseils, Bob et le diagnostic photo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="153" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="153" t="inlineStr">
+        <is>
+          <t>Ajout validé par Jordan : badge « Gardien de l'hiver » (onglet Badges &amp; Objectifs) et règle de notification de la Ligue d'hiver (onglet Règles Notifications).</t>
         </is>
       </c>
     </row>

</xml_diff>